<commit_message>
Facility Yield Analysis: base case → V2-vintage ≥90 DPD loss (C); lifetime ≥90 kept as conservative sensitivity
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -45,7 +45,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +67,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -99,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +124,8 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -510,6 +515,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -588,7 +594,6 @@
           <t>KPI Dashboard Monthly r52, Sep 2026</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -609,7 +614,6 @@
           <t>KPI Dashboard Monthly r53, Sep 2026</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -630,7 +634,6 @@
           <t>KPI Dashboard Monthly r49, Sep 2026</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -973,7 +976,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Base case: fully seasoned 'has gone bad' measure</t>
+          <t>Conservative case: fully seasoned 'has gone bad' measure across all vintages incl. V1-model 2025</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1026,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Lags the &gt;15 column by construction on young vintages</t>
+          <t>BASE CASE (Steve, 2026-10-26): V2 model from Dec 2025; go-forward baseline. Young vintages — will rise with seasoning; &gt;15 DPD for the same window is 1.559%</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1106,6 @@
           <t>KPI Dashboard Monthly r84, Sep 2026</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1187,6 +1189,30 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1198,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1215,6 +1241,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1380,8 +1407,8 @@
         <f>C9*12</f>
         <v/>
       </c>
-      <c r="E9" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1434,7 +1461,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>A. Lifetime vintage loss, ≥90 DPD (base case)</t>
+          <t>A. Lifetime vintage loss, ≥90 DPD (conservative)</t>
         </is>
       </c>
       <c r="B14" s="8">
@@ -1482,7 +1509,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C. V2-model vintages since Jan 2026, ≥90 DPD (lower)</t>
+          <t>C. V2-model vintages since Jan 2026, ≥90 DPD (BASE CASE)</t>
         </is>
       </c>
       <c r="B16" s="8">
@@ -1499,7 +1526,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Young vintages; will rise with seasoning — a floor, not a forecast</t>
+          <t>Base case per Steve 2026-10-26: V2 model rolled out Dec 2025 with a visible break in delinquency; treated as the go-forward baseline. Caveat: vintages ≤9 months old — the ≥90 DPD rate will rise as they season (the &gt;15 DPD rate for the same window is 1.56%).</t>
         </is>
       </c>
     </row>
@@ -1528,10 +1555,11 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>NET YIELD AND EXCESS SPREAD (base case = loss A)</t>
+          <t>NET YIELD AND EXCESS SPREAD (base case = loss C, V2 vintages)</t>
         </is>
       </c>
     </row>
@@ -1568,20 +1596,19 @@
         <f>D9</f>
         <v/>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>− Loss on receivables (A)</t>
+          <t>− Loss on receivables (C, V2 vintages)</t>
         </is>
       </c>
       <c r="B22" s="9">
-        <f>D14</f>
+        <f>D16</f>
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>D14</f>
+        <f>D16</f>
         <v/>
       </c>
       <c r="E22" t="inlineStr">
@@ -1603,7 +1630,6 @@
         <f>C21-C22</f>
         <v/>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1644,6 +1670,26 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Sensitivity: excess spread at the conservative lifetime ≥90 DPD loss (A)</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>B25-(D14-D16)</f>
+        <v/>
+      </c>
+      <c r="C26" s="18">
+        <f>C25-(D14-D16)</f>
+        <v/>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Difference between A and C is the entire V1→V2 narrative; a lender will ask for both</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
@@ -1754,6 +1800,33 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1765,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1780,6 +1853,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -1811,6 +1885,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1857,11 +1932,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>− Loss on receivables (base case A)</t>
+          <t>− Loss on receivables (base case C, V2 vintages)</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>'Today — Sep 2026'!D14</f>
+        <f>'Today — Sep 2026'!D16</f>
         <v/>
       </c>
     </row>
@@ -1896,6 +1971,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
@@ -1910,6 +1986,16 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1921,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1950,6 +2036,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2034,6 +2121,8 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
@@ -2236,6 +2325,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
@@ -2437,6 +2527,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -2638,13 +2729,46 @@
         <v/>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Read across: the base case (today's share, lifetime ≥90 DPD, 19%) reproduces the Today sheet. Moving to 50–55% revolving adds 2–4 points of gross yield; the V2-vintage loss rate adds ~3–4 points; each 2 points of coupon is worth 1.6 points of excess spread at an 80% advance.</t>
-        </is>
-      </c>
-    </row>
+          <t>Read across: base case = today's share, V2 ≥90 DPD loss (first loss column), 19% coupon — 8.9 points of excess spread; the lifetime columns show the conservative case a lender will also run. Moving to 50–55% revolving adds ~1–1.5 points; each 2 points of coupon is worth 1.6 points at an 80% advance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>

</xml_diff>

<commit_message>
Facility Yield Analysis: fix label cells Excel parsed as formulas (repair dialog, #NAME?); verified via LibreOffice recalculation, no error cells
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -679,9 +679,10 @@
           <t>KPI Dashboard Monthly r40, Sep 2026</t>
         </is>
       </c>
-      <c r="E11">
-        <f> sum of the five lines above</f>
-        <v/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sum of the five lines above</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1189,30 +1190,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1224,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1432,9 +1409,10 @@
           <t>× annual originations ÷ avg receivables (turnover)</t>
         </is>
       </c>
-      <c r="D12" s="3">
-        <f> annualized loss on receivables</f>
-        <v/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>annualized loss on receivables</t>
+        </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
@@ -1618,9 +1596,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4">
-        <f> Net yield (before servicing/opex)</f>
-        <v/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>⇒ Net yield (before servicing/opex)</t>
+        </is>
       </c>
       <c r="B23" s="12">
         <f>B21-B22</f>
@@ -1652,9 +1631,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4">
-        <f> Excess spread</f>
-        <v/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>⇒ Excess spread</t>
+        </is>
       </c>
       <c r="B25" s="12">
         <f>B23-B24</f>
@@ -1800,33 +1780,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1838,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1920,9 +1873,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
-        <f> Balance-driven gross yield</f>
-        <v/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>⇒ Balance-driven gross yield</t>
+        </is>
       </c>
       <c r="B12" s="12">
         <f>'Today — Sep 2026'!D7</f>
@@ -1941,9 +1895,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
-        <f> Net collateral yield</f>
-        <v/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>⇒ Net collateral yield</t>
+        </is>
       </c>
       <c r="B14" s="12">
         <f>B12-B13</f>
@@ -1962,9 +1917,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
-        <f> Excess spread, collateral only</f>
-        <v/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>⇒ Excess spread, collateral only</t>
+        </is>
       </c>
       <c r="B16" s="12">
         <f>B14-B15</f>
@@ -1986,16 +1942,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2007,7 +1953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2737,38 +2683,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
@@ -2797,6 +2711,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Copy cited warehouse report snapshots (vintage loss, revolver/transactor) into Analyses (internal)/source-reports with README; workbook paths updated
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -758,7 +758,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>revolver_transactor_balances_2026-01_to_2026-09_10262026.csv, all_revolving, 2026-09</t>
+          <t>source-reports/revolver_transactor_balances_2026-01_to_2026-09_10262026.csv, all_revolving, 2026-09</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>vintage_loss_by_origination_month_10262026.csv, originated_principal_php, 2026-09</t>
+          <t>source-reports/vintage_loss_by_origination_month_10262026.csv, originated_principal_php, 2026-09</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>vintage_loss_since_origination_month_10262026.csv, since 2024-01, loss_rate_16dpd_seasoned_pct = 1.781%</t>
+          <t>source-reports/vintage_loss_since_origination_month_10262026.csv, since 2024-01, loss_rate_16dpd_seasoned_pct = 1.781%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1190,6 +1190,30 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1218,7 +1242,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1385,7 +1408,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1533,7 +1555,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1806,7 +1827,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -1838,7 +1858,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1927,7 +1946,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
@@ -1982,7 +2000,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2067,8 +2084,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
@@ -2271,7 +2286,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
@@ -2473,7 +2487,6 @@
         <v/>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -2675,7 +2688,6 @@
         <v/>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2732,7 +2744,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>~/apps/zed/Analysis+Reports/. Regenerate: bash ~/.claude/skills/revolver-transactor-report/scripts/run_report.sh --from 2026-01 --to 2026-09 (BigQuery epicac-2.zed_reporting views; definitions in the skill). Statement-based: revolving = ending balance less installment charge on statements with interest_charged &gt; 0.</t>
+          <t>Copies in debt_dd/Analyses (internal)/source-reports/ (originals in ~/apps/zed/Analysis+Reports/). Regenerate: bash ~/.claude/skills/revolver-transactor-report/scripts/run_report.sh --from 2026-01 --to 2026-09 (BigQuery epicac-2.zed_reporting views; definitions in the skill). Statement-based: revolving = ending balance less installment charge on statements with interest_charged &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2756,7 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>~/apps/zed/Analysis+Reports/. Regenerate: bash ~/.claude/skills/vintage-loss-report/scripts/run_report.sh (FIFO waterfall views in epicac-2.zed_reporting). Run of 2026-10-26: waterfall vs actual 97.0% exact, 1.35% residual — PASS; delinquent-book tie 0.17% — PASS.</t>
+          <t>Copies in debt_dd/Analyses (internal)/source-reports/ (originals in ~/apps/zed/Analysis+Reports/). Regenerate: bash ~/.claude/skills/vintage-loss-report/scripts/run_report.sh (FIFO waterfall views in epicac-2.zed_reporting). Run of 2026-10-26: waterfall vs actual 97.0% exact, 1.35% residual — PASS; delinquent-book tie 0.17% — PASS.</t>
         </is>
       </c>
     </row>
@@ -2796,6 +2808,16 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Facility Yield Analysis: interchange is inside pledged collections (₱98 funded / ₱100 billed) — replace 'Collateral-only view' with 'Interchange and the lender'; correct yield note
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Today — Sep 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collateral-only view" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interchange and the lender" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +126,15 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -515,7 +524,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1190,30 +1198,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1242,6 +1226,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1361,7 +1346,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Everything a lender sees in pledged collections</t>
+          <t>Revenue that accrues on balances while they sit: billed on statements, paid into the collection account</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1370,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Settled by Mastercard to Zed at T+1 on the merchant side; not a cardholder payment</t>
+          <t>Earned when the receivable is CREATED: Zed funds ₱98 to the merchant via Mastercard and books/bills ₱100. The cardholder's ₱100 lands in the collection account, so the margin is inside pledged collections — realized at origination, not accrued over the balance's life</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1392,13 @@
         <f>C9*12</f>
         <v/>
       </c>
-    </row>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>The lender's coverage measure: everything collected on the pledged pool less what it cost to create</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1555,6 +1546,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1566,12 +1558,12 @@
       <c r="A20" s="3" t="inlineStr"/>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Balance-driven view (collateral only)</t>
+          <t>Accrual-only view (billed interest &amp; fees)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>All-revenue view (incl. interchange)</t>
+          <t>Full collections view (incl. interchange embedded in receivable face) — lender's coverage</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr"/>
@@ -1667,7 +1659,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Negative in the collateral-only view: the facility is being underwritten on interchange + corporate recourse</t>
+          <t>Negative in the accrual-only column only because that column ignores the origination margin; it is NOT a collateral shortfall — see the 'Interchange and the lender' tab</t>
         </is>
       </c>
     </row>
@@ -1812,151 +1804,233 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Why the collateral-only view is 8.2% net — and why it matters for structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>In configuration A (parent borrows; ZFPI grants a lien over the receivables pool + control of the collection account), the lender's security is the cash cardholders pay against their statements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Cardholder payments = statement balance = purchases + revolving interest + installment interest + upfront fees + late fees. The revenue inside those payments is the three interest/fee lines — 'balance-driven yield'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Interchange is paid by Mastercard to Zed at settlement (T+1), netted against what Zed funds to the merchant. It is never billed to a cardholder and never enters the collection account. A lender can only count it through recourse to Zed (guarantee / corporate covenant), not through the pledged asset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="8" customHeight="1">
-      <c r="A6" s="14" t="inlineStr"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Collateral-only arithmetic (Sep 2026, annualized on avg receivables):</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Revolving interest</t>
-        </is>
-      </c>
-      <c r="B9" s="9">
-        <f>'Today — Sep 2026'!D4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Installment interest + upfront fees</t>
-        </is>
-      </c>
-      <c r="B10" s="9">
-        <f>'Today — Sep 2026'!D5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Late fees</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>'Today — Sep 2026'!D6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>⇒ Balance-driven gross yield</t>
-        </is>
-      </c>
-      <c r="B12" s="12">
-        <f>'Today — Sep 2026'!D7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>− Loss on receivables (base case C, V2 vintages)</t>
-        </is>
-      </c>
-      <c r="B13" s="9">
-        <f>'Today — Sep 2026'!D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>⇒ Net collateral yield</t>
-        </is>
-      </c>
-      <c r="B14" s="12">
-        <f>B12-B13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>− Cost of funds (coupon × advance)</t>
-        </is>
-      </c>
-      <c r="B15" s="9">
-        <f>coupon*advance</f>
-        <v/>
-      </c>
+          <t>How interchange reaches the lender — and why the full-collections column is the lender's coverage measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Worked example: a ₱100 purchase at 2% interchange.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>1. Mastercard instructs Zed to settle ₱98 to the merchant (face less interchange). Zed funds the ₱98 at T+1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>2. Zed books a ₱100 receivable and bills the cardholder ₱100 on the next statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>3. The cardholder pays ₱100 into the collection account the lender controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>The ₱2 is therefore inside pledged collections: it is the excess of what is collected on the receivable over what it cost to create. It is realized at origination, so on a yield-on-balances basis it scales with turnover (~11× a year today), not with how long balances sit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="20" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Consequences for the facility:</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>• A lender advancing 80% of face is funding ₱80 of a receivable that cost ₱98; Zed's equity funds ₱18, and the ₱2 margin arrives with the ₱100 of collections. The pool is over-collateralized by the interchange margin on every new receivable.</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>• The lender's coverage test is the full-collections column on the Today sheet (gross 33.6%, net 24.0% at the V2 loss base, 8.8 points over a 19% coupon at 80% advance). The accrual-only column (interest and fees that accrue while a balance sits) is a decomposition, not a collateral boundary.</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>• What is genuinely outside the receivables, and what a first-facility guarantee is compensating for: no borrower/servicer track record, Zed's operational control of settlement and collections, and model risk on young vintages — not interchange.</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>• Interchange would leave the lender's reach only in a true sale priced at face, or if settlement funding ran through accounts outside the structure. In the secured-loan configurations under discussion it is in.</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="19" t="inlineStr"/>
+      <c r="B14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Earlier drafts of this workbook (and the 2026-10-26 yield note) treated interchange as a separate cash stream that bypassed the collection account and showed a negative 'collateral-only' excess spread. That was wrong; corrected 2026-10-26 per Steve.</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>⇒ Excess spread, collateral only</t>
-        </is>
-      </c>
-      <c r="B16" s="12">
-        <f>B14-B15</f>
-        <v/>
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation of the two Today columns (annualized on avg receivables)</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Reading: on pledged cash flows alone, today's book does not carry a high-teens coupon. The facility is therefore underwritten on interchange plus corporate recourse — which is why the parent guarantee is not negotiable away on a first facility, and why negotiation capital is better spent on the coupon.</t>
+          <t>Gross yield</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Accrual-only</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Full collections</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>The All-revenue column on the Today sheet is the same arithmetic with interchange included.</t>
+          <t>Gross yield</t>
+        </is>
+      </c>
+      <c r="B19" s="9">
+        <f>'Today — Sep 2026'!D7</f>
+        <v/>
+      </c>
+      <c r="C19" s="9">
+        <f>'Today — Sep 2026'!D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>of which interchange (origination margin)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="9">
+        <f>'Today — Sep 2026'!D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>− Loss (base case C)</t>
+        </is>
+      </c>
+      <c r="B21" s="9">
+        <f>'Today — Sep 2026'!D16</f>
+        <v/>
+      </c>
+      <c r="C21" s="9">
+        <f>'Today — Sep 2026'!D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>⇒ Net yield</t>
+        </is>
+      </c>
+      <c r="B22" s="9">
+        <f>B19-B21</f>
+        <v/>
+      </c>
+      <c r="C22" s="9">
+        <f>C19-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>− Cost of funds (coupon × advance)</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>coupon*advance</f>
+        <v/>
+      </c>
+      <c r="C23" s="9">
+        <f>coupon*advance</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>⇒ Excess spread</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>B22-B23</f>
+        <v/>
+      </c>
+      <c r="C24" s="9">
+        <f>C22-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>The lender reads the Full collections column. The accrual-only column answers a different question — what the book earns per peso-month it is outstanding — and is the number that rises as revolving share rises.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2723,7 +2797,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -2808,16 +2881,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Facility Yield Analysis: tidy reconciliation header on the interchange tab
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +133,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1226,7 +1229,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1398,7 +1400,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1546,7 +1547,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -1820,6 +1820,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -1922,9 +1923,9 @@
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Gross yield</t>
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Reconciliation of the two Today columns (annualized on avg receivables)</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2027,6 +2028,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="21" t="inlineStr">
         <is>
@@ -2034,6 +2036,19 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Facility Yield Analysis: bucket view — interchange on whole book, not the transacting bucket; note corrected
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1229,6 +1229,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1400,6 +1401,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1547,6 +1549,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1686,7 +1689,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>BUCKET VIEW (monthly yield on each bucket's own balance — reconciles to Steve's BOE sheet)</t>
+          <t>BUCKET VIEW (monthly yield each bucket earns on its own balance — billed interest and fees only)</t>
         </is>
       </c>
     </row>
@@ -1708,12 +1711,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Revenue on this bucket, PHP/mo</t>
+          <t>Billed revenue on this bucket, PHP/mo</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Monthly yield on own balance</t>
+          <t>Monthly yield on own balance (accrual)</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1769,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Transacting (interchange only)</t>
+          <t>Transacting</t>
         </is>
       </c>
       <c r="B31" s="7">
@@ -1777,9 +1780,8 @@
         <f>B31/bal_tot</f>
         <v/>
       </c>
-      <c r="D31" s="7">
-        <f>interchange</f>
-        <v/>
+      <c r="D31" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E31" s="8">
         <f>D31/B31</f>
@@ -1789,10 +1791,58 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Note: interchange is earned on spend, not balances; 3.15%/mo on the transacting bucket only because those balances turn ~2.3× a month. On the whole book it is 1.26%/mo.</t>
-        </is>
-      </c>
-    </row>
+          <t>Interchange — whole book (earned on ALL purchases: transactor spend, revolver spend and installment-converted purchases)</t>
+        </is>
+      </c>
+      <c r="B32" s="7">
+        <f>bal_tot</f>
+        <v/>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7">
+        <f>interchange</f>
+        <v/>
+      </c>
+      <c r="E32" s="8">
+        <f>D32/B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Note: interchange cannot be assigned to one bucket from these reports — it is earned at purchase, and those purchases end up in all three balances. Attributing it all to transacting (as the BOE layout does) overstates that bucket's yield; attributing by spend would need purchases split by revolver/transactor/installment user from the warehouse. On the whole book it is 1.26%/mo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1804,7 +1854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -1820,7 +1870,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -2028,7 +2077,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="21" t="inlineStr">
         <is>
@@ -2036,19 +2084,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Facility Yield Analysis: note distinguishes interchange yield on book (1.26%/mo) from KPI-sheet rate on purchase volume (1.38%)
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261026.xlsx
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1229,7 +1229,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1401,7 +1400,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1549,7 +1547,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1813,36 +1810,10 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Note: interchange cannot be assigned to one bucket from these reports — it is earned at purchase, and those purchases end up in all three balances. Attributing it all to transacting (as the BOE layout does) overstates that bucket's yield; attributing by spend would need purchases split by revolver/transactor/installment user from the warehouse. On the whole book it is 1.26%/mo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+          <t>Note: interchange cannot be assigned to one bucket from these reports — it is earned at purchase, and those purchases end up in all three balances. Attributing it all to transacting (as the BOE layout does) overstates that bucket's yield; attributing by spend would need purchases split by revolver/transactor/installment user from the warehouse. On the whole book it is 1.26%/mo. Not to be confused with the KPI-sheet interchange rate (1.38% for Sep), which divides the same ₱2.63M by purchase/settlement volume (₱191M), not by receivables.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>